<commit_message>
serving the rest of the pages.
</commit_message>
<xml_diff>
--- a/biomed_inventory_app/app/data/pm_completion_report.xlsx
+++ b/biomed_inventory_app/app/data/pm_completion_report.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="completion" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="completion" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:AU1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -440,16 +440,41 @@
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="9" customWidth="1" min="21" max="21"/>
-    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="23" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="23" customWidth="1" min="24" max="24"/>
+    <col width="23" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="19" customWidth="1" min="29" max="29"/>
+    <col width="25" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="17" customWidth="1" min="32" max="32"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="17" customWidth="1" min="35" max="35"/>
+    <col width="19" customWidth="1" min="36" max="36"/>
+    <col width="17" customWidth="1" min="37" max="37"/>
+    <col width="15" customWidth="1" min="38" max="38"/>
+    <col width="24" customWidth="1" min="39" max="39"/>
+    <col width="18" customWidth="1" min="40" max="40"/>
+    <col width="23" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="14" customWidth="1" min="45" max="45"/>
+    <col width="9" customWidth="1" min="46" max="46"/>
+    <col width="17" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -515,50 +540,175 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>client_id</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>department_id</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>equipment_id</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>contract_id</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>case_id</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>scheduled_date</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>assigned_engineer_id</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>pm_label</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>communication_stage</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>reminder_1_sent</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>reminder_2_sent</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>final_reminder_sent</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>engineer_alert_sent</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>visit_confirmed_date</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>overdue</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>source_row_hash</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
           <t>parent_case_reference</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>parent_case_id</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>department_id</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>report_status</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>checklist_status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>blocked_reason</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>blocked_notes</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>client_informed</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>date_informed</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>informed_by</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>communication_method</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>informed_notes</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>informed_attachment</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>asset_tag</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>hospital</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>serial_number</t>
         </is>

</xml_diff>